<commit_message>
changed plot info to match previous version
</commit_message>
<xml_diff>
--- a/inputs/location_code_crosswalk_water_quality.xlsx
+++ b/inputs/location_code_crosswalk_water_quality.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/fnufferrodriguez_usbr_gov/Documents/Desktop/eis-appendix-generation/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="71" documentId="11_F25DC773A252ABDACC10488FF19C59685ADE58F8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{82E20AED-070C-402E-95BA-99F1B1C2EC1A}"/>
+  <xr:revisionPtr revIDLastSave="72" documentId="11_F25DC773A252ABDACC10488FF19C59685ADE58F8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3B522FBC-398B-4DB4-A01D-23DA36C4C53A}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="75" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="38">
   <si>
     <t>Location (Title)</t>
   </si>
@@ -105,9 +105,6 @@
   </si>
   <si>
     <t>RSAN032_AG</t>
-  </si>
-  <si>
-    <t>CHDMC006_AG</t>
   </si>
   <si>
     <t>SLCBN002_FWS</t>
@@ -500,10 +497,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>37</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -511,7 +508,7 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C2" t="s">
         <v>18</v>
@@ -528,7 +525,7 @@
         <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C3" t="s">
         <v>19</v>
@@ -545,7 +542,7 @@
         <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C4" t="s">
         <v>20</v>
@@ -562,7 +559,7 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C5" t="s">
         <v>21</v>
@@ -579,7 +576,7 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C6" t="s">
         <v>22</v>
@@ -596,16 +593,16 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C7" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D7">
-        <v>-1</v>
+        <v>-0.4</v>
       </c>
       <c r="E7">
-        <v>0.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -613,10 +610,10 @@
         <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D8">
         <v>-20</v>
@@ -630,10 +627,10 @@
         <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D9">
         <v>-20</v>
@@ -647,10 +644,10 @@
         <v>13</v>
       </c>
       <c r="B10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D10">
         <v>-20</v>
@@ -664,10 +661,10 @@
         <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D11">
         <v>-20</v>
@@ -681,10 +678,10 @@
         <v>8</v>
       </c>
       <c r="B12" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D12">
         <v>-0.35</v>
@@ -698,10 +695,10 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C13" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D13">
         <v>-0.35</v>
@@ -715,10 +712,10 @@
         <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C14" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D14">
         <v>-20</v>
@@ -732,10 +729,10 @@
         <v>17</v>
       </c>
       <c r="B15" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D15">
         <v>-250</v>
@@ -749,10 +746,10 @@
         <v>4</v>
       </c>
       <c r="B16" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D16">
         <v>-300</v>
@@ -766,10 +763,10 @@
         <v>3</v>
       </c>
       <c r="B17" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C17" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D17">
         <v>-300</v>
@@ -783,10 +780,10 @@
         <v>5</v>
       </c>
       <c r="B18" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C18" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D18">
         <v>-300</v>
@@ -800,10 +797,10 @@
         <v>6</v>
       </c>
       <c r="B19" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C19" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D19">
         <v>-250</v>

</xml_diff>